<commit_message>
Added new sensitivity analyses and formatted VIF table
</commit_message>
<xml_diff>
--- a/notebooks/extra_tables/ema_rwd_final_statistics_tables_logit_formated.xlsx
+++ b/notebooks/extra_tables/ema_rwd_final_statistics_tables_logit_formated.xlsx
@@ -474,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R49"/>
+  <dimension ref="A1:R68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -637,7 +637,7 @@
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>Study required by a Risk Management Plan</t>
+          <t>Study required by an RMP</t>
         </is>
       </c>
       <c r="B5" s="1" t="inlineStr">
@@ -1057,20 +1057,20 @@
     <row r="11">
       <c r="A11" s="1" t="inlineStr">
         <is>
-          <t>Type of funding source</t>
+          <t>Study required by a regulatory body</t>
         </is>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>Commercial</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1785</v>
+        <v>1255</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1085 (60.8)</t>
+          <t>698 (55.6)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr"/>
@@ -1080,11 +1080,11 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
-        <v>1160</v>
+        <v>789</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>840 (72.4)</t>
+          <t>495 (62.7)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr"/>
@@ -1098,403 +1098,363 @@
       <c r="A12" s="1" t="n"/>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Non-Commercial</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>391</v>
+        <v>1021</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>219 (56.0)</t>
+          <t>659 (64.5)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>0.82</t>
+          <t>1.45</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>0.66 - 1.02</t>
+          <t>1.23 - 1.72</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.081</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>0.99</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0.73 - 1.35</t>
-        </is>
-      </c>
-      <c r="J12" t="n">
-        <v>0.961</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
-        <v>246</v>
+        <v>675</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>149 (60.6)</t>
+          <t>516 (76.4)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>0.59</t>
+          <t>1.93</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.44 - 0.78</t>
+          <t>1.53 - 2.42</t>
         </is>
       </c>
       <c r="O12" t="n">
         <v>0</v>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>0.62</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>0.40 - 0.95</t>
-        </is>
-      </c>
-      <c r="R12" t="n">
-        <v>0.028</v>
-      </c>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n"/>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>Mixed</t>
+          <t>Unspecified</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>33 (55.0)</t>
+          <t>13 (54.2)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.79</t>
+          <t>0.94</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>0.47 - 1.32</t>
+          <t>0.42 - 2.12</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.368</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>0.83</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>0.43 - 1.60</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>0.569</v>
-      </c>
+        <v>0.887</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
-        <v>40</v>
+        <v>18</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>13 (32.5)</t>
+          <t>3 (16.7)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>0.18</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.09 - 0.36</t>
+          <t>0.03 - 0.41</t>
         </is>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>0.46</t>
-        </is>
-      </c>
-      <c r="Q13" t="inlineStr">
-        <is>
-          <t>0.20 - 1.08</t>
-        </is>
-      </c>
-      <c r="R13" t="n">
-        <v>0.073</v>
-      </c>
+        <v>0.001</v>
+      </c>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="1" t="n"/>
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Type of funding source</t>
+        </is>
+      </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>Unclear</t>
+          <t>Commercial</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>36</v>
+        <v>1785</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>15 (41.7)</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>0.46</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>0.24 - 0.90</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>0.023</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>0.49</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>0.23 - 1.02</t>
-        </is>
-      </c>
-      <c r="J14" t="n">
-        <v>0.056</v>
-      </c>
+          <t>1085 (60.8)</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="n">
-        <v>22</v>
+        <v>1160</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>7 (31.8)</t>
-        </is>
-      </c>
-      <c r="M14" t="inlineStr">
-        <is>
-          <t>0.18</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>0.07 - 0.44</t>
-        </is>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>0.18</t>
-        </is>
-      </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>0.07 - 0.47</t>
-        </is>
-      </c>
-      <c r="R14" t="n">
-        <v>0</v>
-      </c>
+          <t>840 (72.4)</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n"/>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>No Funding</t>
+          <t>Non-Commercial</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>28</v>
+        <v>391</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>18 (64.3)</t>
+          <t>219 (56.0)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>0.82</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>0.53 - 2.53</t>
+          <t>0.66 - 1.02</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>0.707</v>
+        <v>0.081</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>2.15</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0.91 - 5.06</t>
+          <t>0.73 - 1.35</t>
         </is>
       </c>
       <c r="J15" t="n">
-        <v>0.079</v>
+        <v>0.961</v>
       </c>
       <c r="K15" t="n">
-        <v>14</v>
+        <v>246</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>5 (35.7)</t>
+          <t>149 (60.6)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>0.21</t>
+          <t>0.59</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.07 - 0.64</t>
+          <t>0.44 - 0.78</t>
         </is>
       </c>
       <c r="O15" t="n">
-        <v>0.006</v>
+        <v>0</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.27</t>
+          <t>0.62</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>0.08 - 0.85</t>
+          <t>0.40 - 0.95</t>
         </is>
       </c>
       <c r="R15" t="n">
-        <v>0.025</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>Multiple funding sources</t>
-        </is>
-      </c>
+      <c r="A16" s="1" t="n"/>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Mixed</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2065</v>
+        <v>60</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1244 (60.2)</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+          <t>33 (55.0)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>0.79</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>0.47 - 1.32</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>0.368</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>0.83</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.43 - 1.60</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0.569</v>
+      </c>
       <c r="K16" t="n">
-        <v>1347</v>
+        <v>40</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>953 (70.7)</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr"/>
-      <c r="O16" t="inlineStr"/>
-      <c r="P16" t="inlineStr"/>
-      <c r="Q16" t="inlineStr"/>
-      <c r="R16" t="inlineStr"/>
+          <t>13 (32.5)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>0.18</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0.09 - 0.36</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>0.46</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>0.20 - 1.08</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>0.073</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n"/>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>235</v>
+        <v>36</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>126 (53.6)</t>
+          <t>15 (41.7)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.76</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.58 - 1.00</t>
+          <t>0.24 - 0.90</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>0.05</v>
+        <v>0.023</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>0.77</t>
+          <t>0.49</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>0.55 - 1.10</t>
+          <t>0.23 - 1.02</t>
         </is>
       </c>
       <c r="J17" t="n">
-        <v>0.149</v>
+        <v>0.056</v>
       </c>
       <c r="K17" t="n">
-        <v>135</v>
+        <v>22</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>61 (45.2)</t>
+          <t>7 (31.8)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>0.34</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.24 - 0.49</t>
+          <t>0.07 - 0.44</t>
         </is>
       </c>
       <c r="O17" t="n">
@@ -1502,12 +1462,12 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0.39</t>
+          <t>0.18</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>0.25 - 0.63</t>
+          <t>0.07 - 0.47</t>
         </is>
       </c>
       <c r="R17" t="n">
@@ -1515,178 +1475,178 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1" t="inlineStr">
-        <is>
-          <t>Number of PAS funded by sponsor, quartiles</t>
-        </is>
-      </c>
+      <c r="A18" s="1" t="n"/>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>No Funding</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>519</v>
+        <v>28</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>348 (67.1)</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+          <t>18 (64.3)</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.16</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.53 - 2.53</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0.707</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2.15</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>0.91 - 5.06</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>0.079</v>
+      </c>
       <c r="K18" t="n">
-        <v>326</v>
+        <v>14</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>286 (87.7)</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr"/>
-      <c r="O18" t="inlineStr"/>
-      <c r="P18" t="inlineStr"/>
-      <c r="Q18" t="inlineStr"/>
-      <c r="R18" t="inlineStr"/>
+          <t>5 (35.7)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>0.21</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0.07 - 0.64</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>0.27</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>0.08 - 0.85</t>
+        </is>
+      </c>
+      <c r="R18" t="n">
+        <v>0.025</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="1" t="n"/>
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>Multiple funding sources</t>
+        </is>
+      </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>No</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>611</v>
+        <v>2065</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>293 (48.0)</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>0.45</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>0.36 - 0.58</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>0.56</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>0.43 - 0.74</t>
-        </is>
-      </c>
-      <c r="J19" t="n">
-        <v>0</v>
-      </c>
+          <t>1244 (60.2)</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
       <c r="K19" t="n">
-        <v>373</v>
+        <v>1347</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>191 (51.2)</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr">
-        <is>
-          <t>0.15</t>
-        </is>
-      </c>
-      <c r="N19" t="inlineStr">
-        <is>
-          <t>0.10 - 0.22</t>
-        </is>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="inlineStr">
-        <is>
-          <t>0.08</t>
-        </is>
-      </c>
-      <c r="Q19" t="inlineStr">
-        <is>
-          <t>0.05 - 0.13</t>
-        </is>
-      </c>
-      <c r="R19" t="n">
-        <v>0</v>
-      </c>
+          <t>953 (70.7)</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr"/>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr"/>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n"/>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>604</v>
+        <v>235</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>349 (57.8)</t>
+          <t>126 (53.6)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0.67</t>
+          <t>0.76</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0.53 - 0.86</t>
+          <t>0.58 - 1.00</t>
         </is>
       </c>
       <c r="G20" t="n">
-        <v>0.001</v>
+        <v>0.05</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0.75</t>
+          <t>0.77</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>0.56 - 0.99</t>
+          <t>0.55 - 1.10</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>0.039</v>
+        <v>0.149</v>
       </c>
       <c r="K20" t="n">
-        <v>390</v>
+        <v>135</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>259 (66.4)</t>
+          <t>61 (45.2)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>0.28</t>
+          <t>0.34</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.19 - 0.41</t>
+          <t>0.24 - 0.49</t>
         </is>
       </c>
       <c r="O20" t="n">
@@ -1694,12 +1654,12 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0.20</t>
+          <t>0.39</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>0.12 - 0.32</t>
+          <t>0.25 - 0.63</t>
         </is>
       </c>
       <c r="R20" t="n">
@@ -1707,178 +1667,178 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="1" t="n"/>
+      <c r="A21" s="1" t="inlineStr">
+        <is>
+          <t>Number of PAS funded by sponsor, quartiles</t>
+        </is>
+      </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>566</v>
+        <v>519</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>380 (67.1)</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>1.00</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>0.78 - 1.29</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>0.976</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>0.89 - 1.60</t>
-        </is>
-      </c>
-      <c r="J21" t="n">
-        <v>0.23</v>
-      </c>
+          <t>348 (67.1)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
       <c r="K21" t="n">
-        <v>393</v>
+        <v>326</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>278 (70.7)</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>0.34</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>0.23 - 0.50</t>
-        </is>
-      </c>
-      <c r="O21" t="n">
+          <t>286 (87.7)</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr"/>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n"/>
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>611</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>293 (48.0)</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0.36 - 0.58</t>
+        </is>
+      </c>
+      <c r="G22" t="n">
         <v>0</v>
       </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>0.30</t>
-        </is>
-      </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>0.18 - 0.49</t>
-        </is>
-      </c>
-      <c r="R21" t="n">
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>0.56</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>0.43 - 0.74</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="1" t="inlineStr">
-        <is>
-          <t>Countries in which study is conducted</t>
-        </is>
-      </c>
-      <c r="B22" s="1" t="inlineStr">
-        <is>
-          <t>Single Country</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>1355</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>759 (56.0)</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
       <c r="K22" t="n">
-        <v>905</v>
+        <v>373</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>574 (63.4)</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
+          <t>191 (51.2)</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0.10 - 0.22</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>0.08</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>0.05 - 0.13</t>
+        </is>
+      </c>
+      <c r="R22" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n"/>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>Multiple Countries</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>945</v>
+        <v>604</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>611 (64.7)</t>
+          <t>349 (57.8)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.44</t>
+          <t>0.67</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1.21 - 1.70</t>
+          <t>0.53 - 0.86</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.31</t>
+          <t>0.75</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1.06 - 1.62</t>
+          <t>0.56 - 0.99</t>
         </is>
       </c>
       <c r="J23" t="n">
-        <v>0.011</v>
+        <v>0.039</v>
       </c>
       <c r="K23" t="n">
-        <v>577</v>
+        <v>390</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>440 (76.3)</t>
+          <t>259 (66.4)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>0.28</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>1.46 - 2.34</t>
+          <t>0.19 - 0.41</t>
         </is>
       </c>
       <c r="O23" t="n">
@@ -1886,227 +1846,227 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>1.35</t>
+          <t>0.20</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>1.01 - 1.80</t>
+          <t>0.12 - 0.32</t>
         </is>
       </c>
       <c r="R23" t="n">
-        <v>0.045</v>
+        <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr">
-        <is>
-          <t>Study type</t>
-        </is>
-      </c>
+      <c r="A24" s="1" t="n"/>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>Non-interventional</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2224</v>
+        <v>566</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1344 (60.4)</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr"/>
+          <t>380 (67.1)</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>0.78 - 1.29</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>0.89 - 1.60</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>0.23</v>
+      </c>
       <c r="K24" t="n">
-        <v>1438</v>
+        <v>393</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>990 (68.8)</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+          <t>278 (70.7)</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>0.34</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0.23 - 0.50</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>0.18 - 0.49</t>
+        </is>
+      </c>
+      <c r="R24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n"/>
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>Countries in which study is conducted</t>
+        </is>
+      </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>Clinical trial</t>
+          <t>Single Country</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>32</v>
+        <v>1355</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10 (31.2)</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>0.30</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>0.14 - 0.63</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>0.33</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>0.14 - 0.77</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>0.01</v>
-      </c>
+          <t>759 (56.0)</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr"/>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
       <c r="K25" t="n">
-        <v>21</v>
+        <v>905</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>12 (57.1)</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>0.60</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr">
-        <is>
-          <t>0.25 - 1.44</t>
-        </is>
-      </c>
-      <c r="O25" t="n">
-        <v>0.256</v>
-      </c>
-      <c r="P25" t="inlineStr">
-        <is>
-          <t>0.86</t>
-        </is>
-      </c>
-      <c r="Q25" t="inlineStr">
-        <is>
-          <t>0.30 - 2.48</t>
-        </is>
-      </c>
-      <c r="R25" t="n">
-        <v>0.783</v>
-      </c>
+          <t>574 (63.4)</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr"/>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n"/>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>Not applicable</t>
+          <t>Multiple Countries</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>44</v>
+        <v>945</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>16 (36.4)</t>
+          <t>611 (64.7)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0.37</t>
+          <t>1.44</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>0.20 - 0.70</t>
+          <t>1.21 - 1.70</t>
         </is>
       </c>
       <c r="G26" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0.43</t>
+          <t>1.31</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>0.22 - 0.87</t>
+          <t>1.06 - 1.62</t>
         </is>
       </c>
       <c r="J26" t="n">
-        <v>0.019</v>
+        <v>0.011</v>
       </c>
       <c r="K26" t="n">
-        <v>23</v>
+        <v>577</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>12 (52.2)</t>
+          <t>440 (76.3)</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>0.49</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>0.22 - 1.13</t>
+          <t>1.46 - 2.34</t>
         </is>
       </c>
       <c r="O26" t="n">
-        <v>0.094</v>
+        <v>0</v>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>0.53</t>
+          <t>1.35</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>0.20 - 1.45</t>
+          <t>1.01 - 1.80</t>
         </is>
       </c>
       <c r="R26" t="n">
-        <v>0.217</v>
+        <v>0.045</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="inlineStr">
         <is>
-          <t>Estimated total number of subjects</t>
+          <t>Study type</t>
         </is>
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>100-&lt;500</t>
+          <t>Non-interventional</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>498</v>
+        <v>2224</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>279 (56.0)</t>
+          <t>1344 (60.4)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr"/>
@@ -2116,11 +2076,11 @@
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
       <c r="K27" t="n">
-        <v>320</v>
+        <v>1438</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>230 (71.9)</t>
+          <t>990 (68.8)</t>
         </is>
       </c>
       <c r="M27" t="inlineStr"/>
@@ -2134,515 +2094,515 @@
       <c r="A28" s="1" t="n"/>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>&lt;100</t>
+          <t>Clinical trial</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>260</v>
+        <v>32</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>155 (59.6)</t>
+          <t>10 (31.2)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.16</t>
+          <t>0.30</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>0.85 - 1.57</t>
+          <t>0.14 - 0.63</t>
         </is>
       </c>
       <c r="G28" t="n">
-        <v>0.343</v>
+        <v>0.002</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>0.33</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>0.95 - 1.88</t>
+          <t>0.14 - 0.77</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>0.096</v>
+        <v>0.01</v>
       </c>
       <c r="K28" t="n">
-        <v>168</v>
+        <v>21</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>123 (73.2)</t>
+          <t>12 (57.1)</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>0.60</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>0.70 - 1.63</t>
+          <t>0.25 - 1.44</t>
         </is>
       </c>
       <c r="O28" t="n">
-        <v>0.753</v>
+        <v>0.256</v>
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>0.99</t>
+          <t>0.86</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
         <is>
-          <t>0.61 - 1.61</t>
+          <t>0.30 - 2.48</t>
         </is>
       </c>
       <c r="R28" t="n">
-        <v>0.971</v>
+        <v>0.783</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n"/>
       <c r="B29" s="1" t="inlineStr">
         <is>
-          <t>500-&lt;1000</t>
+          <t>Not applicable</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>244</v>
+        <v>44</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>140 (57.4)</t>
+          <t>16 (36.4)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.06</t>
+          <t>0.37</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>0.78 - 1.44</t>
+          <t>0.20 - 0.70</t>
         </is>
       </c>
       <c r="G29" t="n">
-        <v>0.727</v>
+        <v>0.002</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>0.43</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>0.72 - 1.41</t>
+          <t>0.22 - 0.87</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>0.971</v>
+        <v>0.019</v>
       </c>
       <c r="K29" t="n">
-        <v>146</v>
+        <v>23</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>92 (63.0)</t>
+          <t>12 (52.2)</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>0.67</t>
+          <t>0.49</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>0.44 - 1.01</t>
+          <t>0.22 - 1.13</t>
         </is>
       </c>
       <c r="O29" t="n">
-        <v>0.056</v>
+        <v>0.094</v>
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>0.68</t>
+          <t>0.53</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
         <is>
-          <t>0.42 - 1.09</t>
+          <t>0.20 - 1.45</t>
         </is>
       </c>
       <c r="R29" t="n">
-        <v>0.106</v>
+        <v>0.217</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1" t="n"/>
+      <c r="A30" s="1" t="inlineStr">
+        <is>
+          <t>Estimated total number of subjects</t>
+        </is>
+      </c>
       <c r="B30" s="1" t="inlineStr">
         <is>
-          <t>1000-10000</t>
+          <t>100-&lt;500</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>569</v>
+        <v>498</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>329 (57.8)</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>1.08</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>0.84 - 1.37</t>
-        </is>
-      </c>
-      <c r="G30" t="n">
-        <v>0.554</v>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>1.14</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>0.87 - 1.49</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>0.354</v>
-      </c>
+          <t>279 (56.0)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
       <c r="K30" t="n">
-        <v>347</v>
+        <v>320</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>232 (66.9)</t>
-        </is>
-      </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>0.79</t>
-        </is>
-      </c>
-      <c r="N30" t="inlineStr">
-        <is>
-          <t>0.57 - 1.10</t>
-        </is>
-      </c>
-      <c r="O30" t="n">
-        <v>0.161</v>
-      </c>
-      <c r="P30" t="inlineStr">
-        <is>
-          <t>0.74</t>
-        </is>
-      </c>
-      <c r="Q30" t="inlineStr">
-        <is>
-          <t>0.50 - 1.08</t>
-        </is>
-      </c>
-      <c r="R30" t="n">
-        <v>0.121</v>
-      </c>
+          <t>230 (71.9)</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n"/>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>&gt;10000</t>
+          <t>&lt;100</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>729</v>
+        <v>260</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>467 (64.1)</t>
+          <t>155 (59.6)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.40</t>
+          <t>1.16</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>1.11 - 1.77</t>
+          <t>0.85 - 1.57</t>
         </is>
       </c>
       <c r="G31" t="n">
-        <v>0.005</v>
+        <v>0.343</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>1.34</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>1.03 - 1.85</t>
+          <t>0.95 - 1.88</t>
         </is>
       </c>
       <c r="J31" t="n">
-        <v>0.03</v>
+        <v>0.096</v>
       </c>
       <c r="K31" t="n">
-        <v>501</v>
+        <v>168</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>337 (67.3)</t>
+          <t>123 (73.2)</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>1.07</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>0.59 - 1.09</t>
+          <t>0.70 - 1.63</t>
         </is>
       </c>
       <c r="O31" t="n">
-        <v>0.164</v>
+        <v>0.753</v>
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>0.84</t>
+          <t>0.99</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
         <is>
-          <t>0.57 - 1.24</t>
+          <t>0.61 - 1.61</t>
         </is>
       </c>
       <c r="R31" t="n">
-        <v>0.378</v>
+        <v>0.971</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1" t="inlineStr">
-        <is>
-          <t>Age of study population</t>
-        </is>
-      </c>
+      <c r="A32" s="1" t="n"/>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>≥18 years</t>
+          <t>500-&lt;1000</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1467</v>
+        <v>244</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>850 (57.9)</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr"/>
-      <c r="G32" t="inlineStr"/>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+          <t>140 (57.4)</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.06</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>0.78 - 1.44</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>0.727</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>0.72 - 1.41</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>0.971</v>
+      </c>
       <c r="K32" t="n">
-        <v>955</v>
+        <v>146</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>652 (68.3)</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
+          <t>92 (63.0)</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>0.67</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0.44 - 1.01</t>
+        </is>
+      </c>
+      <c r="O32" t="n">
+        <v>0.056</v>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>0.68</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>0.42 - 1.09</t>
+        </is>
+      </c>
+      <c r="R32" t="n">
+        <v>0.106</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n"/>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>&lt;18 years</t>
+          <t>1000-10000</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>148</v>
+        <v>569</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>89 (60.1)</t>
+          <t>329 (57.8)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.10</t>
+          <t>1.08</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>0.78 - 1.55</t>
+          <t>0.84 - 1.37</t>
         </is>
       </c>
       <c r="G33" t="n">
-        <v>0.606</v>
+        <v>0.554</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>1.02</t>
+          <t>1.14</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>0.69 - 1.49</t>
+          <t>0.87 - 1.49</t>
         </is>
       </c>
       <c r="J33" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.354</v>
       </c>
       <c r="K33" t="n">
-        <v>99</v>
+        <v>347</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>64 (64.6)</t>
+          <t>232 (66.9)</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>0.85</t>
+          <t>0.79</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>0.55 - 1.31</t>
+          <t>0.57 - 1.10</t>
         </is>
       </c>
       <c r="O33" t="n">
-        <v>0.462</v>
+        <v>0.161</v>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>1.37</t>
+          <t>0.74</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>0.81 - 2.30</t>
+          <t>0.50 - 1.08</t>
         </is>
       </c>
       <c r="R33" t="n">
-        <v>0.242</v>
+        <v>0.121</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n"/>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>&lt;18 and ≥18 years</t>
+          <t>&gt;10000</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>685</v>
+        <v>729</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>431 (62.9)</t>
+          <t>467 (64.1)</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>1.40</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>1.02 - 1.48</t>
+          <t>1.11 - 1.77</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>0.029</v>
+        <v>0.005</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1.15</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>0.92 - 1.42</t>
+          <t>1.03 - 1.85</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>0.221</v>
+        <v>0.03</v>
       </c>
       <c r="K34" t="n">
-        <v>428</v>
+        <v>501</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>298 (69.6)</t>
+          <t>337 (67.3)</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>1.07</t>
+          <t>0.80</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>0.83 - 1.36</t>
+          <t>0.59 - 1.09</t>
         </is>
       </c>
       <c r="O34" t="n">
-        <v>0.616</v>
+        <v>0.164</v>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>1.34</t>
+          <t>0.84</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>0.99 - 1.82</t>
+          <t>0.57 - 1.24</t>
         </is>
       </c>
       <c r="R34" t="n">
-        <v>0.058</v>
+        <v>0.378</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="inlineStr">
         <is>
-          <t>Medical condition(s) to be studied</t>
+          <t>Age of study population</t>
         </is>
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>≥18 years</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1668</v>
+        <v>1467</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>995 (59.7)</t>
+          <t>850 (57.9)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -2652,11 +2612,11 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr"/>
       <c r="K35" t="n">
-        <v>1080</v>
+        <v>955</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>747 (69.2)</t>
+          <t>652 (68.3)</t>
         </is>
       </c>
       <c r="M35" t="inlineStr"/>
@@ -2670,503 +2630,535 @@
       <c r="A36" s="1" t="n"/>
       <c r="B36" s="1" t="inlineStr">
         <is>
+          <t>&lt;18 years</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>148</v>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>89 (60.1)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.10</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>0.78 - 1.55</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>0.606</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>1.02</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>0.69 - 1.49</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>0.9330000000000001</v>
+      </c>
+      <c r="K36" t="n">
+        <v>99</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>64 (64.6)</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0.55 - 1.31</t>
+        </is>
+      </c>
+      <c r="O36" t="n">
+        <v>0.462</v>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>1.37</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>0.81 - 2.30</t>
+        </is>
+      </c>
+      <c r="R36" t="n">
+        <v>0.242</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="n"/>
+      <c r="B37" s="1" t="inlineStr">
+        <is>
+          <t>&lt;18 and ≥18 years</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>685</v>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>431 (62.9)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>1.02 - 1.48</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>0.92 - 1.42</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>0.221</v>
+      </c>
+      <c r="K37" t="n">
+        <v>428</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>298 (69.6)</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>1.07</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0.83 - 1.36</t>
+        </is>
+      </c>
+      <c r="O37" t="n">
+        <v>0.616</v>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>0.99 - 1.82</t>
+        </is>
+      </c>
+      <c r="R37" t="n">
+        <v>0.058</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr">
+        <is>
+          <t>Medical condition(s) to be studied</t>
+        </is>
+      </c>
+      <c r="B38" s="1" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>1668</v>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>995 (59.7)</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="n">
+        <v>1080</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>747 (69.2)</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr"/>
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="n"/>
+      <c r="B39" s="1" t="inlineStr">
+        <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C36" t="n">
+      <c r="C39" t="n">
         <v>632</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>375 (59.3)</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>0.99</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>0.82 - 1.19</t>
         </is>
       </c>
-      <c r="G36" t="n">
+      <c r="G39" t="n">
         <v>0.89</v>
       </c>
-      <c r="H36" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>0.97</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>0.78 - 1.21</t>
         </is>
       </c>
-      <c r="J36" t="n">
+      <c r="J39" t="n">
         <v>0.797</v>
       </c>
-      <c r="K36" t="n">
+      <c r="K39" t="n">
         <v>402</v>
       </c>
-      <c r="L36" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>267 (66.4)</t>
         </is>
       </c>
-      <c r="M36" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>0.88</t>
         </is>
       </c>
-      <c r="N36" t="inlineStr">
+      <c r="N39" t="inlineStr">
         <is>
           <t>0.69 - 1.13</t>
         </is>
       </c>
-      <c r="O36" t="n">
+      <c r="O39" t="n">
         <v>0.312</v>
       </c>
-      <c r="P36" t="inlineStr">
+      <c r="P39" t="inlineStr">
         <is>
           <t>0.86</t>
         </is>
       </c>
-      <c r="Q36" t="inlineStr">
+      <c r="Q39" t="inlineStr">
         <is>
           <t>0.64 - 1.16</t>
         </is>
       </c>
-      <c r="R36" t="n">
+      <c r="R39" t="n">
         <v>0.329</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr">
         <is>
           <t>Outcomes specified</t>
         </is>
       </c>
-      <c r="B37" s="1" t="inlineStr">
+      <c r="B40" s="1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C37" t="n">
+      <c r="C40" t="n">
         <v>381</v>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>231 (60.6)</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="n">
+      <c r="E40" t="inlineStr"/>
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="n">
         <v>274</v>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L40" t="inlineStr">
         <is>
           <t>166 (60.6)</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="n"/>
-      <c r="B38" s="1" t="inlineStr">
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr"/>
+      <c r="O40" t="inlineStr"/>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="n"/>
+      <c r="B41" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C38" t="n">
+      <c r="C41" t="n">
         <v>1919</v>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>1139 (59.4)</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>0.95</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F41" t="inlineStr">
         <is>
           <t>0.76 - 1.19</t>
         </is>
       </c>
-      <c r="G38" t="n">
+      <c r="G41" t="n">
         <v>0.643</v>
       </c>
-      <c r="H38" t="inlineStr">
+      <c r="H41" t="inlineStr">
         <is>
           <t>1.08</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="I41" t="inlineStr">
         <is>
           <t>0.83 - 1.40</t>
         </is>
       </c>
-      <c r="J38" t="n">
+      <c r="J41" t="n">
         <v>0.556</v>
       </c>
-      <c r="K38" t="n">
+      <c r="K41" t="n">
         <v>1208</v>
       </c>
-      <c r="L38" t="inlineStr">
+      <c r="L41" t="inlineStr">
         <is>
           <t>848 (70.2)</t>
         </is>
       </c>
-      <c r="M38" t="inlineStr">
+      <c r="M41" t="inlineStr">
         <is>
           <t>1.53</t>
         </is>
       </c>
-      <c r="N38" t="inlineStr">
+      <c r="N41" t="inlineStr">
         <is>
           <t>1.17 - 2.01</t>
         </is>
       </c>
-      <c r="O38" t="n">
+      <c r="O41" t="n">
         <v>0.002</v>
       </c>
-      <c r="P38" t="inlineStr">
+      <c r="P41" t="inlineStr">
         <is>
           <t>1.76</t>
         </is>
       </c>
-      <c r="Q38" t="inlineStr">
+      <c r="Q41" t="inlineStr">
         <is>
           <t>1.26 - 2.46</t>
         </is>
       </c>
-      <c r="R38" t="n">
+      <c r="R41" t="n">
         <v>0.001</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr">
         <is>
           <t>Collaboration of a research network</t>
         </is>
       </c>
-      <c r="B39" s="1" t="inlineStr">
+      <c r="B42" s="1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="C42" t="n">
         <v>2039</v>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>1185 (58.1)</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr"/>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
-      <c r="I39" t="inlineStr"/>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="n">
+      <c r="E42" t="inlineStr"/>
+      <c r="F42" t="inlineStr"/>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="n">
         <v>1338</v>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L42" t="inlineStr">
         <is>
           <t>928 (69.4)</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="n"/>
-      <c r="B40" s="1" t="inlineStr">
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr"/>
+      <c r="O42" t="inlineStr"/>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="n"/>
+      <c r="B43" s="1" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C40" t="n">
+      <c r="C43" t="n">
         <v>261</v>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D43" t="inlineStr">
         <is>
           <t>185 (70.9)</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E43" t="inlineStr">
         <is>
           <t>1.75</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F43" t="inlineStr">
         <is>
           <t>1.32 - 2.32</t>
         </is>
       </c>
-      <c r="G40" t="n">
+      <c r="G43" t="n">
         <v>0</v>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H43" t="inlineStr">
         <is>
           <t>2.19</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I43" t="inlineStr">
         <is>
           <t>1.57 - 3.05</t>
         </is>
       </c>
-      <c r="J40" t="n">
+      <c r="J43" t="n">
         <v>0</v>
       </c>
-      <c r="K40" t="n">
+      <c r="K43" t="n">
         <v>144</v>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="L43" t="inlineStr">
         <is>
           <t>86 (59.7)</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="M43" t="inlineStr">
         <is>
           <t>0.66</t>
         </is>
       </c>
-      <c r="N40" t="inlineStr">
+      <c r="N43" t="inlineStr">
         <is>
           <t>0.46 - 0.93</t>
         </is>
       </c>
-      <c r="O40" t="n">
+      <c r="O43" t="n">
         <v>0.019</v>
       </c>
-      <c r="P40" t="inlineStr">
+      <c r="P43" t="inlineStr">
         <is>
           <t>0.63</t>
         </is>
       </c>
-      <c r="Q40" t="inlineStr">
+      <c r="Q43" t="inlineStr">
         <is>
           <t>0.40 - 0.97</t>
         </is>
       </c>
-      <c r="R40" t="n">
+      <c r="R43" t="n">
         <v>0.037</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr">
         <is>
           <t>Study uses established data source</t>
         </is>
       </c>
-      <c r="B41" s="1" t="inlineStr">
+      <c r="B44" s="1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C41" t="n">
+      <c r="C44" t="n">
         <v>1558</v>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D44" t="inlineStr">
         <is>
           <t>885 (56.8)</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="n">
+      <c r="E44" t="inlineStr"/>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="n">
         <v>981</v>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L44" t="inlineStr">
         <is>
           <t>684 (69.7)</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="n"/>
-      <c r="B42" s="1" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C42" t="n">
-        <v>742</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>485 (65.4)</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>1.44</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>1.20 - 1.72</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>0.96 - 1.51</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>0.116</v>
-      </c>
-      <c r="K42" t="n">
-        <v>501</v>
-      </c>
-      <c r="L42" t="inlineStr">
-        <is>
-          <t>330 (65.9)</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr">
-        <is>
-          <t>0.84</t>
-        </is>
-      </c>
-      <c r="N42" t="inlineStr">
-        <is>
-          <t>0.67 - 1.05</t>
-        </is>
-      </c>
-      <c r="O42" t="n">
-        <v>0.131</v>
-      </c>
-      <c r="P42" t="inlineStr">
-        <is>
-          <t>0.83</t>
-        </is>
-      </c>
-      <c r="Q42" t="inlineStr">
-        <is>
-          <t>0.61 - 1.12</t>
-        </is>
-      </c>
-      <c r="R42" t="n">
-        <v>0.223</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr">
-        <is>
-          <t>Status of study</t>
-        </is>
-      </c>
-      <c r="B43" s="1" t="inlineStr">
-        <is>
-          <t>Finalised</t>
-        </is>
-      </c>
-      <c r="C43" t="n">
-        <v>1484</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>1030 (69.4)</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
-      <c r="G43" t="inlineStr"/>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
-      <c r="K43" t="inlineStr"/>
-      <c r="L43" t="inlineStr"/>
-      <c r="M43" t="inlineStr"/>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
-      <c r="P43" t="inlineStr"/>
-      <c r="Q43" t="inlineStr"/>
-      <c r="R43" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="n"/>
-      <c r="B44" s="1" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>816</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>340 (41.7)</t>
-        </is>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>0.31</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>0.26 - 0.38</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>0.23</t>
-        </is>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>0.18 - 0.29</t>
-        </is>
-      </c>
-      <c r="J44" t="n">
-        <v>0</v>
-      </c>
-      <c r="K44" t="inlineStr"/>
-      <c r="L44" t="inlineStr"/>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
       <c r="O44" t="inlineStr"/>
@@ -3175,202 +3167,174 @@
       <c r="R44" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="inlineStr">
-        <is>
-          <t>Planned duration of study, quartiles</t>
-        </is>
-      </c>
+      <c r="A45" s="1" t="n"/>
       <c r="B45" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>460</v>
+        <v>742</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>296 (64.3)</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr"/>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
+          <t>485 (65.4)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.44</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>1.20 - 1.72</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>0.96 - 1.51</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>0.116</v>
+      </c>
       <c r="K45" t="n">
-        <v>297</v>
+        <v>501</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>198 (66.7)</t>
-        </is>
-      </c>
-      <c r="M45" t="inlineStr"/>
-      <c r="N45" t="inlineStr"/>
-      <c r="O45" t="inlineStr"/>
-      <c r="P45" t="inlineStr"/>
-      <c r="Q45" t="inlineStr"/>
-      <c r="R45" t="inlineStr"/>
+          <t>330 (65.9)</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>0.84</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0.67 - 1.05</t>
+        </is>
+      </c>
+      <c r="O45" t="n">
+        <v>0.131</v>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>0.83</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>0.61 - 1.12</t>
+        </is>
+      </c>
+      <c r="R45" t="n">
+        <v>0.223</v>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="n"/>
+      <c r="A46" s="1" t="inlineStr">
+        <is>
+          <t>Status of study</t>
+        </is>
+      </c>
       <c r="B46" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Finalised</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>462</v>
+        <v>1484</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>298 (64.5)</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>1.01</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>0.77 - 1.32</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>0.961</v>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>1.20</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>0.89 - 1.62</t>
-        </is>
-      </c>
-      <c r="J46" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="K46" t="n">
-        <v>293</v>
-      </c>
-      <c r="L46" t="inlineStr">
-        <is>
-          <t>204 (69.6)</t>
-        </is>
-      </c>
-      <c r="M46" t="inlineStr">
-        <is>
-          <t>1.15</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>0.81 - 1.62</t>
-        </is>
-      </c>
-      <c r="O46" t="n">
-        <v>0.441</v>
-      </c>
-      <c r="P46" t="inlineStr">
-        <is>
-          <t>1.09</t>
-        </is>
-      </c>
-      <c r="Q46" t="inlineStr">
-        <is>
-          <t>0.73 - 1.62</t>
-        </is>
-      </c>
-      <c r="R46" t="n">
-        <v>0.6860000000000001</v>
-      </c>
+          <t>1030 (69.4)</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr"/>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr"/>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n"/>
       <c r="B47" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Ongoing</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>457</v>
+        <v>816</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>257 (56.2)</t>
+          <t>340 (41.7)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.31</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>0.55 - 0.93</t>
+          <t>0.26 - 0.38</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>0.012</v>
+        <v>0</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>0.98</t>
+          <t>0.23</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>0.72 - 1.33</t>
+          <t>0.18 - 0.29</t>
         </is>
       </c>
       <c r="J47" t="n">
-        <v>0.894</v>
-      </c>
-      <c r="K47" t="n">
-        <v>294</v>
-      </c>
-      <c r="L47" t="inlineStr">
-        <is>
-          <t>204 (69.4)</t>
-        </is>
-      </c>
-      <c r="M47" t="inlineStr">
-        <is>
-          <t>1.13</t>
-        </is>
-      </c>
-      <c r="N47" t="inlineStr">
-        <is>
-          <t>0.80 - 1.60</t>
-        </is>
-      </c>
-      <c r="O47" t="n">
-        <v>0.478</v>
-      </c>
-      <c r="P47" t="inlineStr">
-        <is>
-          <t>1.12</t>
-        </is>
-      </c>
-      <c r="Q47" t="inlineStr">
-        <is>
-          <t>0.75 - 1.69</t>
-        </is>
-      </c>
-      <c r="R47" t="n">
-        <v>0.573</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K47" t="inlineStr"/>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr"/>
+      <c r="N47" t="inlineStr"/>
+      <c r="O47" t="inlineStr"/>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
+      <c r="R47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="n"/>
+      <c r="A48" s="1" t="inlineStr">
+        <is>
+          <t>Planned duration of study, quartiles</t>
+        </is>
+      </c>
       <c r="B48" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -3378,170 +3342,1225 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>280 (60.9)</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>0.86</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>0.66 - 1.13</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>0.276</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>1.43</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>1.01 - 2.02</t>
-        </is>
-      </c>
-      <c r="J48" t="n">
-        <v>0.042</v>
-      </c>
+          <t>296 (64.3)</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr"/>
       <c r="K48" t="n">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>227 (76.9)</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>1.67</t>
-        </is>
-      </c>
-      <c r="N48" t="inlineStr">
-        <is>
-          <t>1.16 - 2.40</t>
-        </is>
-      </c>
-      <c r="O48" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="P48" t="inlineStr">
-        <is>
-          <t>1.23</t>
-        </is>
-      </c>
-      <c r="Q48" t="inlineStr">
-        <is>
-          <t>0.80 - 1.90</t>
-        </is>
-      </c>
-      <c r="R48" t="n">
-        <v>0.339</v>
-      </c>
+          <t>198 (66.7)</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr"/>
+      <c r="N48" t="inlineStr"/>
+      <c r="O48" t="inlineStr"/>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr"/>
+      <c r="R48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="1" t="n"/>
       <c r="B49" s="1" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>462</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>298 (64.5)</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>0.77 - 1.32</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>0.961</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>1.20</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>0.89 - 1.62</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="K49" t="n">
+        <v>293</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>204 (69.6)</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>1.15</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0.81 - 1.62</t>
+        </is>
+      </c>
+      <c r="O49" t="n">
+        <v>0.441</v>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>0.73 - 1.62</t>
+        </is>
+      </c>
+      <c r="R49" t="n">
+        <v>0.6860000000000001</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="n"/>
+      <c r="B50" s="1" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>457</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>257 (56.2)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>0.71</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>0.55 - 0.93</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>0.012</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>0.98</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>0.72 - 1.33</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>0.894</v>
+      </c>
+      <c r="K50" t="n">
+        <v>294</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>204 (69.4)</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>1.13</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0.80 - 1.60</t>
+        </is>
+      </c>
+      <c r="O50" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="P50" t="inlineStr">
+        <is>
+          <t>1.12</t>
+        </is>
+      </c>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>0.75 - 1.69</t>
+        </is>
+      </c>
+      <c r="R50" t="n">
+        <v>0.573</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="n"/>
+      <c r="B51" s="1" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>460</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>280 (60.9)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>0.66 - 1.13</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>0.276</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>1.43</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>1.01 - 2.02</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="K51" t="n">
+        <v>295</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>227 (76.9)</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>1.67</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>1.16 - 2.40</t>
+        </is>
+      </c>
+      <c r="O51" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="P51" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="Q51" t="inlineStr">
+        <is>
+          <t>0.80 - 1.90</t>
+        </is>
+      </c>
+      <c r="R51" t="n">
+        <v>0.339</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1" t="n"/>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
           <t>Unspecified</t>
         </is>
       </c>
-      <c r="C49" t="n">
+      <c r="C52" t="n">
         <v>461</v>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D52" t="inlineStr">
         <is>
           <t>239 (51.8)</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E52" t="inlineStr">
         <is>
           <t>0.60</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F52" t="inlineStr">
         <is>
           <t>0.46 - 0.78</t>
         </is>
       </c>
-      <c r="G49" t="n">
+      <c r="G52" t="n">
         <v>0</v>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="H52" t="inlineStr">
         <is>
           <t>0.82</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
+      <c r="I52" t="inlineStr">
         <is>
           <t>0.60 - 1.12</t>
         </is>
       </c>
-      <c r="J49" t="n">
+      <c r="J52" t="n">
         <v>0.216</v>
       </c>
-      <c r="K49" t="n">
+      <c r="K52" t="n">
         <v>303</v>
       </c>
-      <c r="L49" t="inlineStr">
+      <c r="L52" t="inlineStr">
         <is>
           <t>181 (59.7)</t>
         </is>
       </c>
-      <c r="M49" t="inlineStr">
+      <c r="M52" t="inlineStr">
         <is>
           <t>0.74</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr">
+      <c r="N52" t="inlineStr">
         <is>
           <t>0.53 - 1.03</t>
         </is>
       </c>
-      <c r="O49" t="n">
+      <c r="O52" t="n">
         <v>0.079</v>
       </c>
-      <c r="P49" t="inlineStr">
+      <c r="P52" t="inlineStr">
         <is>
           <t>0.67</t>
         </is>
       </c>
-      <c r="Q49" t="inlineStr">
+      <c r="Q52" t="inlineStr">
         <is>
           <t>0.45 - 0.99</t>
         </is>
       </c>
-      <c r="R49" t="n">
+      <c r="R52" t="n">
         <v>0.044</v>
       </c>
     </row>
+    <row r="53">
+      <c r="A53" s="1" t="inlineStr">
+        <is>
+          <t>registration_year_grouped</t>
+        </is>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>2010-2013</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>189</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>116 (61.4)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr"/>
+      <c r="K53" t="n">
+        <v>153</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>99 (64.7)</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr"/>
+      <c r="N53" t="inlineStr"/>
+      <c r="O53" t="inlineStr"/>
+      <c r="P53" t="inlineStr"/>
+      <c r="Q53" t="inlineStr"/>
+      <c r="R53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n"/>
+      <c r="B54" s="1" t="inlineStr">
+        <is>
+          <t>2014</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>228</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>127 (55.7)</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>0.79</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>0.53 - 1.17</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>0.242</v>
+      </c>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr"/>
+      <c r="K54" t="n">
+        <v>195</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>137 (70.3)</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>0.82 - 2.02</t>
+        </is>
+      </c>
+      <c r="O54" t="n">
+        <v>0.272</v>
+      </c>
+      <c r="P54" t="inlineStr"/>
+      <c r="Q54" t="inlineStr"/>
+      <c r="R54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="n"/>
+      <c r="B55" s="1" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>214</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>131 (61.2)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>0.99</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>0.66 - 1.48</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>0.974</v>
+      </c>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr"/>
+      <c r="K55" t="n">
+        <v>173</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>113 (65.3)</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>1.03</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>0.65 - 1.62</t>
+        </is>
+      </c>
+      <c r="O55" t="n">
+        <v>0.908</v>
+      </c>
+      <c r="P55" t="inlineStr"/>
+      <c r="Q55" t="inlineStr"/>
+      <c r="R55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="n"/>
+      <c r="B56" s="1" t="inlineStr">
+        <is>
+          <t>2016</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>257</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>163 (63.4)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>1.09</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>0.74 - 1.61</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr"/>
+      <c r="K56" t="n">
+        <v>206</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>141 (68.4)</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>0.76 - 1.84</t>
+        </is>
+      </c>
+      <c r="O56" t="n">
+        <v>0.457</v>
+      </c>
+      <c r="P56" t="inlineStr"/>
+      <c r="Q56" t="inlineStr"/>
+      <c r="R56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="n"/>
+      <c r="B57" s="1" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>228</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>155 (68.0)</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>1.34</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>0.89 - 2.00</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr"/>
+      <c r="K57" t="n">
+        <v>178</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>125 (70.2)</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>1.29</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>0.81 - 2.04</t>
+        </is>
+      </c>
+      <c r="O57" t="n">
+        <v>0.285</v>
+      </c>
+      <c r="P57" t="inlineStr"/>
+      <c r="Q57" t="inlineStr"/>
+      <c r="R57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="n"/>
+      <c r="B58" s="1" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>181</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>119 (65.7)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>1.21</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>0.79 - 1.85</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>0.383</v>
+      </c>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr"/>
+      <c r="K58" t="n">
+        <v>113</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>82 (72.6)</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>1.44</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>0.85 - 2.45</t>
+        </is>
+      </c>
+      <c r="O58" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="P58" t="inlineStr"/>
+      <c r="Q58" t="inlineStr"/>
+      <c r="R58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="n"/>
+      <c r="B59" s="1" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>218</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>125 (57.3)</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>0.85</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>0.57 - 1.26</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>0.409</v>
+      </c>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr"/>
+      <c r="J59" t="inlineStr"/>
+      <c r="K59" t="n">
+        <v>123</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>81 (65.9)</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>1.05</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>0.64 - 1.73</t>
+        </is>
+      </c>
+      <c r="O59" t="n">
+        <v>0.842</v>
+      </c>
+      <c r="P59" t="inlineStr"/>
+      <c r="Q59" t="inlineStr"/>
+      <c r="R59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="n"/>
+      <c r="B60" s="1" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>247</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>156 (63.2)</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>1.08</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>0.73 - 1.59</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>0.703</v>
+      </c>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr"/>
+      <c r="K60" t="n">
+        <v>133</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>94 (70.7)</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>1.31</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
+          <t>0.80 - 2.17</t>
+        </is>
+      </c>
+      <c r="O60" t="n">
+        <v>0.283</v>
+      </c>
+      <c r="P60" t="inlineStr"/>
+      <c r="Q60" t="inlineStr"/>
+      <c r="R60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="n"/>
+      <c r="B61" s="1" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>222</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>121 (54.5)</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>0.75</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>0.51 - 1.12</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="H61" t="inlineStr"/>
+      <c r="I61" t="inlineStr"/>
+      <c r="J61" t="inlineStr"/>
+      <c r="K61" t="n">
+        <v>102</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>78 (76.5)</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>1.77</t>
+        </is>
+      </c>
+      <c r="N61" t="inlineStr">
+        <is>
+          <t>1.01 - 3.12</t>
+        </is>
+      </c>
+      <c r="O61" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="P61" t="inlineStr"/>
+      <c r="Q61" t="inlineStr"/>
+      <c r="R61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n"/>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>157</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>72 (45.9)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>0.53</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>0.35 - 0.82</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="H62" t="inlineStr"/>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
+      <c r="K62" t="n">
+        <v>54</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>33 (61.1)</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>0.86</t>
+        </is>
+      </c>
+      <c r="N62" t="inlineStr">
+        <is>
+          <t>0.45 - 1.63</t>
+        </is>
+      </c>
+      <c r="O62" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="P62" t="inlineStr"/>
+      <c r="Q62" t="inlineStr"/>
+      <c r="R62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n"/>
+      <c r="B63" s="1" t="inlineStr">
+        <is>
+          <t>2023-2024</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>159</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>85 (53.5)</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>0.72</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>0.47 - 1.11</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>0.137</v>
+      </c>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr"/>
+      <c r="J63" t="inlineStr"/>
+      <c r="K63" t="n">
+        <v>52</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>31 (59.6)</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>0.81</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>0.42 - 1.54</t>
+        </is>
+      </c>
+      <c r="O63" t="n">
+        <v>0.511</v>
+      </c>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr">
+        <is>
+          <t>study_topic_grouped</t>
+        </is>
+      </c>
+      <c r="B64" s="1" t="inlineStr">
+        <is>
+          <t>Unspecified</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>865</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>380 (43.9)</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr"/>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr"/>
+      <c r="J64" t="inlineStr"/>
+      <c r="K64" t="n">
+        <v>53</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>41 (77.4)</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr"/>
+      <c r="O64" t="inlineStr"/>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="n"/>
+      <c r="B65" s="1" t="inlineStr">
+        <is>
+          <t>Disease /health condition</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>169</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>112 (66.3)</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2.51</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>1.77 - 3.54</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>0</v>
+      </c>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr"/>
+      <c r="J65" t="inlineStr"/>
+      <c r="K65" t="n">
+        <v>169</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>85 (50.3)</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>0.15 - 0.60</t>
+        </is>
+      </c>
+      <c r="O65" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="n"/>
+      <c r="B66" s="1" t="inlineStr">
+        <is>
+          <t>Disease /health condition; Human medicinal product</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>969</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>662 (68.3)</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2.75</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>2.27 - 3.33</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>0</v>
+      </c>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr"/>
+      <c r="J66" t="inlineStr"/>
+      <c r="K66" t="n">
+        <v>964</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>692 (71.8)</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>0.74</t>
+        </is>
+      </c>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>0.39 - 1.44</t>
+        </is>
+      </c>
+      <c r="O66" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="n"/>
+      <c r="B67" s="1" t="inlineStr">
+        <is>
+          <t>Human medicinal product</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>253</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>193 (76.3)</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>4.11</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>2.98 - 5.65</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>0</v>
+      </c>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr"/>
+      <c r="J67" t="inlineStr"/>
+      <c r="K67" t="n">
+        <v>252</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>173 (68.7)</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>0.64</t>
+        </is>
+      </c>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>0.32 - 1.29</t>
+        </is>
+      </c>
+      <c r="O67" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="n"/>
+      <c r="B68" s="1" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>44</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>23 (52.3)</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>1.40</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>0.76 - 2.56</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>0.279</v>
+      </c>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr"/>
+      <c r="J68" t="inlineStr"/>
+      <c r="K68" t="n">
+        <v>44</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>23 (52.3)</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>0.32</t>
+        </is>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>0.13 - 0.77</t>
+        </is>
+      </c>
+      <c r="O68" t="n">
+        <v>0.011</v>
+      </c>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="25">
     <mergeCell ref="P2:R2"/>
-    <mergeCell ref="A41:A42"/>
-    <mergeCell ref="A16:A17"/>
-    <mergeCell ref="A32:A34"/>
+    <mergeCell ref="A14:A18"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="E2:G2"/>
+    <mergeCell ref="A35:A37"/>
     <mergeCell ref="C1:J1"/>
+    <mergeCell ref="A25:A26"/>
     <mergeCell ref="K1:R1"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A21:A24"/>
+    <mergeCell ref="A46:A47"/>
+    <mergeCell ref="A64:A68"/>
+    <mergeCell ref="A48:A52"/>
+    <mergeCell ref="A30:A34"/>
     <mergeCell ref="C2:D2"/>
-    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A53:A63"/>
+    <mergeCell ref="A42:A43"/>
     <mergeCell ref="K2:L2"/>
-    <mergeCell ref="A11:A15"/>
-    <mergeCell ref="A45:A49"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="A19:A20"/>
     <mergeCell ref="A5:A10"/>
-    <mergeCell ref="A35:A36"/>
-    <mergeCell ref="A43:A44"/>
-    <mergeCell ref="A27:A31"/>
-    <mergeCell ref="A39:A40"/>
+    <mergeCell ref="A44:A45"/>
+    <mergeCell ref="A38:A39"/>
+    <mergeCell ref="A40:A41"/>
     <mergeCell ref="M2:O2"/>
+    <mergeCell ref="A27:A29"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>